<commit_message>
feat(F-NAR-019): ATOM-DIF.BES.002-07 La lettre de Mila
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.002-07.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.002-07.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>bureau près du salon, porte de la cuisine</t>
+          <t>bureau près du salon, porte de la cuisine, tiroir, gomme rose, rayon, volet, enveloppe</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mila veut glisser une lettre-soleil sous la porte de la cuisine. Victorina dit non, puis regarder. L'autocollant colle au doigt. Mila accepte, décolle, et papa trouve la lettre.</t>
+          <t>Le tiroir sent le papier. Une gomme rose roule. Un rayon entre par le volet. Sur le rabat, un éclat d'enveloppe luit. Mila veut glisser la lettre-soleil sous la porte, maintenant, avec Victorina. Elle tend trop vite : non, l'autocollant colle, le soleil reste hors. Sourire parti. Elle refuse de foncer, attend le silence, dit d'accord. Merci vécu. Elle pousse d'un coup : l'enveloppe se coince. Elle s'arrête, lit l'éclat. Un éclat d'enveloppe reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le tiroir du bureau sent le papier. Une gomme rose roule. Un rayon entre par le volet. Il fait un rectangle sur le tapis. Une enveloppe jaune attend. Un crayon bleu aussi. Tu as vu le rayon, Mila ? Oui, maman. Il est chaud. Oui. J'épluche les carottes, là. Dans la cuisine. Je veux lui écrire. Une lettre, pour papa ? Oui. En ce moment, Mila prend le crayon. Le bois est lisse. Elle dessine un soleil. Le soleil a des rayons ronds. Il est beau, ce soleil. Il est pour papa. Maman ouvre la porte. Victorina arrive, tout doux. Elle reste près du tapis. Tu viens ? On colle le soleil. Non. Mila écoute. D'accord. On peut proposer. Tu as proposé, Mila. Mila prend un autocollant. Il est rouge, un peu brillant. Il colle à son doigt. Il reste ! Tout doux. Victorina s'assoit près du tapis. Elle regarde le doigt. Tu m'aides ? Je regarde. D'accord. Regarder, c'est une réponse. Le rayon glisse sur la gomme. La gomme est tiède. La soupe sent déjà, ici. Ma lettre aussi. Le crayon roule un peu. Mila le rattrape. Tu as fini de dessiner ? Presque.</t>
+          <t>Le tiroir du bureau sent le papier. Une gomme rose roule, sans bruit. Le bureau est près du salon. Mila connaît ce tiroir, ce bureau. Un rayon entre par le volet. Il est chaud, maman. Tu le sens, sur tes mains ? Oui, un peu. Le rayon fait un rectangle clair. Il tient sur le bureau. J'épluche les carottes, là. Derrière la porte, dans la cuisine. Je t'écris, papa. Une lettre, pour lui ? Oui, maintenant. Une enveloppe jaune attend. Le rabat est un peu luisant. Sur le rabat, un éclat d'enveloppe luit. Il brille, maman ! Tu le vois, sur l'enveloppe ? Oui, près du rabat. Mila touche l'éclat d'enveloppe, un instant. Le papier est lisse, un peu chaud. Elle est tiède. Tu restes près du bureau ? Oui, papa. En ce moment, Mila prend le crayon. Le crayon est lisse, bleu. Elle dessine un soleil. Le soleil a des rayons ronds. Il est beau, ce soleil. Il est pour papa. Maman ouvre la porte de la cuisine. Victorina arrive, près du tapis. Elle reste un moment, les mains collées. Tu viens ? On colle le soleil. Non. Mila tend l'autocollant trop vite. Il colle à son doigt. Il reste ! Tu le prends, maintenant ! Non. Victorina recule d'un pas. Le soleil reste hors de l'enveloppe. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le mets ! L'enveloppe n'est pas fermée. Tu le vois, Mila ? Les épaules de Mila tombent un peu. Ça serre, dans son ventre. Maman se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le tiroir du bureau sent le papier. Une gomme rose roule. Un rayon entre par le volet. Il fait un rectangle sur le tapis. Une enveloppe jaune attend. Un crayon bleu aussi. Tu as vu le rayon, Mila ? Oui, maman. Il est chaud. Oui. J'épluche les carottes, là. Dans la cuisine. Je veux lui écrire. Une lettre, pour papa ? Oui. En ce moment, Mila prend le crayon. Le bois est lisse. Elle dessine un soleil. Le soleil a des rayons ronds. Il est beau, ce soleil. Il est pour papa. Maman ouvre la porte. Victorina arrive, tout doux. Elle reste près du tapis. Tu viens ? On colle le soleil. Non. Mila écoute. D'accord. On peut proposer. Tu as proposé, Mila. Mila prend un autocollant. Il est rouge, un peu brillant. Il colle à son doigt. Il reste ! Tout doux. Victorina s'assoit près du tapis. Elle regarde le doigt. Tu m'aides ? Je regarde. D'accord. Regarder, c'est une réponse. Le rayon glisse sur la gomme. La gomme est tiède. La soupe sent déjà, ici. Ma lettre aussi. Le crayon roule un peu. Mila le rattrape. Tu as fini de dessiner ? Presque.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le tiroir du bureau sent le papier. Une gomme rose roule, sans bruit. Le bureau est près du salon. Mila connaît ce tiroir, ce bureau. Un rayon entre par le volet. Il est chaud, maman. Tu le sens, sur tes mains ? Oui, un peu. Le rayon fait un rectangle clair. Il tient sur le bureau. J'épluche les carottes, là. Derrière la porte, dans la cuisine. Je t'écris, papa. Une lettre, pour lui ? Oui, maintenant. Une enveloppe jaune attend. Le rabat est un peu luisant. Sur le rabat, un &lt;emphasis level="moderate"&gt;éclat d'enveloppe&lt;/emphasis&gt; luit. Il brille, maman ! Tu le vois, sur l'enveloppe ? Oui, près du rabat. Mila touche l'éclat d'enveloppe, un instant. Le papier est lisse, un peu chaud. Elle est tiède. Tu restes près du bureau ? Oui, papa. En ce moment, Mila prend le crayon. Le crayon est lisse, bleu. Elle dessine un soleil. Le soleil a des rayons ronds. Il est beau, ce soleil. Il est pour papa. Maman ouvre la porte de la cuisine. Victorina arrive, près du tapis. Elle reste un moment, les mains collées. Tu viens ? On colle le soleil. Non. Mila tend l'autocollant trop vite. Il colle à son doigt. Il reste ! Tu le prends, maintenant ! Non. Victorina recule d'un pas. Le soleil reste hors de l'enveloppe. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le mets ! L'enveloppe n'est pas fermée. Tu le vois, Mila ? Les épaules de Mila tombent un peu. Ça serre, dans son ventre. Maman se baisse à sa hauteur.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Amandine est à la cuisine. Les petites assiettes sont sur le tapis. Maman ouvre la porte. Nora arrive. Amandine veut jouer. Elle va &lt;emphasis&gt;proposer&lt;/emphasis&gt; un jeu. Amandine dit : tu viens ? Nora dit : non. Amandine regarde maman. Maman dit : on peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. Amandine dit : d'accord. Elle pose une tasse. Nora s'assoit près du buffet. Elle regarde. Amandine laisse Nora à sa place. Elle propose encore, tout doux. Amandine dit : plus tard, tu viens ? Nora dit : je regarde. Maman sourit. Maman dit : regarder, c'est une réponse. On peut accepter plusieurs réponses. Amandine verse de l'eau dans une tasse. Nora avance un peu. Elle ne touche pas. C'est bien. Amandine dit : tu veux une tasse ? Nora dit : plus tard. Amandine dit : d'accord. Elle continue. Maman chante tout bas. Amandine va proposer : on sert le thé. Nora hoche la tête. Elle vient. Elle pose une cuillère. Puis elle s'arrête. Amandine accepte. Elles restent près des tasses. Maman dit : tu as su proposer. Tu as su accepter. Plusieurs réponses sont possibles.&lt;/slow&gt; [pause]</t>
+          <t>Le tiroir du bureau sent le papier. Une gomme rose roule, sans bruit. Le bureau est près du salon. Mila connaît ce tiroir, ce bureau. Un rayon entre par le volet. Il est chaud, maman. Tu le sens, sur tes mains ? Oui, un peu. Le rayon fait un rectangle clair. Il tient sur le bureau. J'épluche les carottes, là. Derrière la porte, dans la cuisine. Je t'écris, papa. Une lettre, pour lui ? Oui, maintenant. Une enveloppe jaune attend. Le rabat est un peu luisant. Sur le rabat, un &lt;emphasis&gt;éclat d'enveloppe&lt;/emphasis&gt; luit. Il brille, maman ! Tu le vois, sur l'enveloppe ? Oui, près du rabat. Mila touche l'éclat d'enveloppe, un instant. Le papier est lisse, un peu chaud. Elle est tiède. Tu restes près du bureau ? Oui, papa. En ce moment, Mila prend le crayon. Le crayon est lisse, bleu. Elle dessine un soleil. Le soleil a des rayons ronds. Il est beau, ce soleil. Il est pour papa. Maman ouvre la porte de la cuisine. Victorina arrive, près du tapis. Elle reste un moment, les mains collées. Tu viens ? On colle le soleil. Non. Mila tend l'autocollant trop vite. Il colle à son doigt. Il reste ! Tu le prends, maintenant ! Non. Victorina recule d'un pas. Le soleil reste hors de l'enveloppe. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le mets ! L'enveloppe n'est pas fermée. Tu le vois, Mila ? Les épaules de Mila tombent un peu. Ça serre, dans son ventre. Maman se baisse à sa hauteur. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>proposer</t>
+          <t>éclat d'enveloppe</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,61 +1324,73 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_lettre_et_victorina_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
           <t>narrateur|Le tiroir du bureau sent le papier.
-narrateur|Une gomme rose roule.
+narrateur|Une gomme rose roule, sans bruit.
+narrateur|Le bureau est près du salon.
+narrateur|Mila connaît ce tiroir, ce bureau.
 narrateur|Un rayon entre par le volet.
-narrateur|Il fait un rectangle sur le tapis.
+enfant-f|Il est chaud, maman.
+maman|Tu le sens, sur tes mains ?
+enfant-f|Oui, un peu.
+narrateur|Le rayon fait un rectangle clair.
+narrateur|Il tient sur le bureau.
+papa|J'épluche les carottes, là.
+papa|Derrière la porte, dans la cuisine.
+enfant-f|Je t'écris, papa.
+maman|Une lettre, pour lui ?
+enfant-f|Oui, maintenant.
 narrateur|Une enveloppe jaune attend.
-narrateur|Un crayon bleu aussi.
-maman|Tu as vu le rayon, Mila ?
-enfant-f|Oui, maman.
-enfant-f|Il est chaud.
-maman|Oui.
-papa|J'épluche les carottes, là.
-papa|Dans la cuisine.
-enfant-f|Je veux lui écrire.
-maman|Une lettre, pour papa ?
-enfant-f|Oui.
+narrateur|Le rabat est un peu luisant.
+narrateur|Sur le rabat, un éclat d'enveloppe luit.
+enfant-f|Il brille, maman !
+maman|Tu le vois, sur l'enveloppe ?
+enfant-f|Oui, près du rabat.
+narrateur|Mila touche l'éclat d'enveloppe, un instant.
+narrateur|Le papier est lisse, un peu chaud.
+enfant-f|Elle est tiède.
+papa|Tu restes près du bureau ?
+enfant-f|Oui, papa.
 narrateur|En ce moment, Mila prend le crayon.
-narrateur|Le bois est lisse.
+narrateur|Le crayon est lisse, bleu.
 narrateur|Elle dessine un soleil.
 narrateur|Le soleil a des rayons ronds.
 maman|Il est beau, ce soleil.
 enfant-f|Il est pour papa.
-narrateur|Maman ouvre la porte.
-narrateur|Victorina arrive, tout doux.
-narrateur|Elle reste près du tapis.
+narrateur|Maman ouvre la porte de la cuisine.
+narrateur|Victorina arrive, près du tapis.
+narrateur|Elle reste un moment, les mains collées.
 enfant-f|Tu viens ?
 enfant-f|On colle le soleil.
 copine|Non.
-narrateur|Mila écoute.
-enfant-f|D'accord.
-maman|On peut proposer.
-maman|Tu as proposé, Mila.
-narrateur|Mila prend un autocollant.
-narrateur|Il est rouge, un peu brillant.
+narrateur|Mila tend l'autocollant trop vite.
 narrateur|Il colle à son doigt.
 enfant-f|Il reste !
-maman|Tout doux.
-narrateur|Victorina s'assoit près du tapis.
-narrateur|Elle regarde le doigt.
-enfant-f|Tu m'aides ?
-copine|Je regarde.
-enfant-f|D'accord.
-maman|Regarder, c'est une réponse.
-narrateur|Le rayon glisse sur la gomme.
-narrateur|La gomme est tiède.
-papa|La soupe sent déjà, ici.
-enfant-f|Ma lettre aussi.
-narrateur|Le crayon roule un peu.
-narrateur|Mila le rattrape.
-maman|Tu as fini de dessiner ?
-enfant-f|Presque.</t>
+enfant-f|Tu le prends, maintenant !
+copine|Non.
+narrateur|Victorina recule d'un pas.
+narrateur|Le soleil reste hors de l'enveloppe.
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-f|Je le mets !
+maman|L'enveloppe n'est pas fermée.
+papa|Tu le vois, Mila ?
+narrateur|Les épaules de Mila tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|Maman se baisse à sa hauteur.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>tiroir,papier</t>
         </is>
       </c>
     </row>
@@ -1410,12 +1422,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Mila invite Victorina. Que fait-on ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Mila invite &lt;emphasis level="moderate"&gt;Victorina&lt;/emphasis&gt;. Que fait-on ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Amandine invite Nora. Que fait-on ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Mila invite &lt;emphasis&gt;Victorina&lt;/emphasis&gt;. Que fait-on ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1440,7 +1452,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On peut proposer. Que fait Mila ?</t>
+          <t>On peut proposer. On peut accepter. Que fait-on ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1478,7 +1490,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1486,10 +1498,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1504,34 +1516,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Victorina</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1540,13 +1556,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1556,7 +1572,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=mila_invite_sans_forcer; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1589,17 +1605,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mila frotte le doigt au bois. L'autocollant se décolle. Il vient ! Oui. On peut accepter plusieurs réponses. Mila pose le soleil dans l'enveloppe. Elle colle le rouge, tout doux. Victorina avance un peu. Elle ne touche pas. Tu veux fermer ? Plus tard. D'accord. Mila glisse l'enveloppe. Elle passe sous la porte. Le papier fait un petit bruit. Il y a une lettre ! C'est le soleil ! Je l'ouvre. La porte s'ouvre un peu. Ça sent la carotte chaude. Le soleil est pour moi ? Oui, papa. Tu as accepté, Mila. Victorina regarde encore. Elle reste près du tapis.</t>
+          <t>Mila avance trop vite vers l'enveloppe. Tu viens, maintenant ! Sa voix se mélange au papier. Oh. Victorina reste près du tapis. Mila refuse de foncer. Elle referme la main. Tu veux venir près du bureau ? Maman s'accroupit à la même hauteur. Mila pose un genou près du tiroir. Tu regardes ? Victorina ne dit rien. Ses mains restent collées. Plus tard, tu viens ? Je regarde. D'accord. Merci, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Mila frotte le doigt au bureau. L'autocollant se décolle. Il vient ! Le soleil est là. Mila pose le soleil dans l'enveloppe. Elle colle le rouge, sans presser. Tu veux fermer ? Plus tard. D'accord. Victorina s'assoit près du tapis. Elle regarde le rabat. Ça sent la carotte, ici. Ma lettre aussi. Le crayon roule un peu. Mila le rattrape. Tu as fini de dessiner ? Presque.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mila frotte le doigt au bois. L'autocollant se décolle. Il vient ! Oui. On peut accepter plusieurs réponses. Mila pose le soleil dans l'enveloppe. Elle colle le rouge, tout doux. Victorina avance un peu. Elle ne touche pas. Tu veux fermer ? Plus tard. D'accord. Mila glisse l'enveloppe. Elle passe sous la porte. Le papier fait un petit bruit. Il y a une lettre ! C'est le soleil ! Je l'ouvre. La porte s'ouvre un peu. Ça sent la carotte chaude. Le soleil est pour moi ? Oui, papa. Tu as accepté, Mila. Victorina regarde encore. Elle reste près du tapis.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila avance trop vite vers l'enveloppe. Tu viens, maintenant ! Sa voix se mélange au papier. Oh. Victorina reste près du tapis. Mila refuse de foncer. Elle referme la main. Tu veux venir près du bureau ? Maman s'accroupit à la même hauteur. Mila pose un genou près du tiroir. Tu regardes ? Victorina ne dit rien. Ses mains restent collées. Plus tard, tu viens ? Je regarde. &lt;emphasis level="moderate"&gt;D'accord&lt;/emphasis&gt;. Merci, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Mila frotte le doigt au bureau. L'autocollant se décolle. Il vient ! Le soleil est là. Mila pose le soleil dans l'enveloppe. Elle colle le rouge, sans presser. Tu veux fermer ? Plus tard. D'accord. Victorina s'assoit près du tapis. Elle regarde le rabat. Ça sent la carotte, ici. Ma lettre aussi. Le crayon roule un peu. Mila le rattrape. Tu as fini de dessiner ? Presque.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Amandine a su &lt;emphasis&gt;proposer&lt;/emphasis&gt;. Nora a dit non, puis regarder. Amandine a pu accepter plusieurs réponses.&lt;/slow&gt; [pause]</t>
+          <t>Mila avance trop vite vers l'enveloppe. Tu viens, maintenant ! Sa voix se mélange au papier. Oh. Victorina reste près du tapis. Mila refuse de foncer. Elle referme la main. Tu veux venir près du bureau ? Maman s'accroupit à la même hauteur. Mila pose un genou près du tiroir. Tu regardes ? Victorina ne dit rien. Ses mains restent collées. Plus tard, tu viens ? Je regarde. &lt;emphasis&gt;D'accord&lt;/emphasis&gt;. Merci, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Mila frotte le doigt au bureau. L'autocollant se décolle. Il vient ! Le soleil est là. Mila pose le soleil dans l'enveloppe. Elle colle le rouge, sans presser. Tu veux fermer ? Plus tard. D'accord. Victorina s'assoit près du tapis. Elle regarde le rabat. Ça sent la carotte, ici. Ma lettre aussi. Le crayon roule un peu. Mila le rattrape. Tu as fini de dessiner ? Presque. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1646,18 +1662,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1680,30 +1696,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>proposer</t>
+          <t>D'accord</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1712,10 +1728,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1724,40 +1740,59 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_attend_le_silence_puis_dit_d_accord; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Mila frotte le doigt au bois.
+          <t>narrateur|Mila avance trop vite vers l'enveloppe.
+enfant-f|Tu viens, maintenant !
+narrateur|Sa voix se mélange au papier.
+enfant-f|Oh.
+narrateur|Victorina reste près du tapis.
+narrateur|Mila refuse de foncer.
+narrateur|Elle referme la main.
+maman|Tu veux venir près du bureau ?
+narrateur|Maman s'accroupit à la même hauteur.
+narrateur|Mila pose un genou près du tiroir.
+enfant-f|Tu regardes ?
+narrateur|Victorina ne dit rien.
+narrateur|Ses mains restent collées.
+enfant-f|Plus tard, tu viens ?
+copine|Je regarde.
+enfant-f|D'accord.
+papa|Merci, Mila.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Mila se desserre.
+narrateur|Les épaules se relèvent un peu.
+maman|Tu as les mains au chaud ?
+enfant-f|Un peu, maman.
+narrateur|Mila frotte le doigt au bureau.
 narrateur|L'autocollant se décolle.
 enfant-f|Il vient !
-maman|Oui.
-maman|On peut accepter plusieurs réponses.
+maman|Le soleil est là.
 narrateur|Mila pose le soleil dans l'enveloppe.
-narrateur|Elle colle le rouge, tout doux.
-narrateur|Victorina avance un peu.
-narrateur|Elle ne touche pas.
+narrateur|Elle colle le rouge, sans presser.
 enfant-f|Tu veux fermer ?
 copine|Plus tard.
 enfant-f|D'accord.
-narrateur|Mila glisse l'enveloppe.
-narrateur|Elle passe sous la porte.
-narrateur|Le papier fait un petit bruit.
-papa|Il y a une lettre !
-enfant-f|C'est le soleil !
-papa|Je l'ouvre.
-narrateur|La porte s'ouvre un peu.
-narrateur|Ça sent la carotte chaude.
-papa|Le soleil est pour moi ?
-enfant-f|Oui, papa.
-maman|Tu as accepté, Mila.
-narrateur|Victorina regarde encore.
-narrateur|Elle reste près du tapis.</t>
+narrateur|Victorina s'assoit près du tapis.
+narrateur|Elle regarde le rabat.
+papa|Ça sent la carotte, ici.
+enfant-f|Ma lettre aussi.
+narrateur|Le crayon roule un peu.
+narrateur|Mila le rattrape.
+maman|Tu as fini de dessiner ?
+enfant-f|Presque.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>papier</t>
         </is>
       </c>
     </row>
@@ -1784,17 +1819,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On range le crayon ? Oui. Mila pose le crayon. Victorina pose la gomme. Le tiroir sent encore le papier. Le soleil est sur la table. Près des carottes. Il brille un peu. Tu as fini de ranger ? Oui, maman. Le rayon a bougé. Il touche maintenant le tapis. La cuisine sent la soupe.</t>
+          <t>Mila pousse l'enveloppe trop vite. Je la glisse, d'un coup ! Le papier se plie sous la porte. L'enveloppe reste coincée. Oh. Le soleil ne passe pas. Je la prends ! Mila avance la main vers Victorina. Tu l'attends, Mila ? Victorina ne bouge pas. Ses mains restent sur ses genoux. Attends, je regarde. Mila s'arrête net. Maman attend, sans parler. Je regarde. Mila observe l'enveloppe, écoute la cuisine. Sur le rabat, un éclat d'enveloppe luit. Là, près du rabat. Mila tient l'enveloppe des deux mains. Le papier est lisse, un peu tiède. Elle est tiède, papa. Tu la portes jusqu'à la porte ? Oui, papa. On avance ? Oui, maman. Mila aplatit le papier, sans forcer. Elle glisse l'enveloppe, très peu. Elle passe. Le rabat aussi, après. Victorina tend la main. Elle pousse un tout petit bord. Il y a une lettre ! C'est le soleil ! Je l'ouvre ? Oui, papa. La porte s'ouvre un peu. Ça sent la carotte chaude. Le soleil est pour moi ? Oui. Mila pose le crayon près du tiroir. Victorina pose la gomme rose.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On range le crayon ? Oui. Mila pose le crayon. Victorina pose la gomme. Le tiroir sent encore le papier. Le soleil est sur la table. Près des carottes. Il brille un peu. Tu as fini de ranger ? Oui, maman. Le rayon a bougé. Il touche maintenant le tapis. La cuisine sent la soupe.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Mila pousse l'enveloppe trop vite. Je la glisse, d'un coup ! Le papier se plie sous la porte. L'enveloppe reste coincée. Oh. Le soleil ne passe pas. Je la prends ! Mila avance la main vers Victorina. Tu l'attends, Mila ? Victorina ne bouge pas. Ses mains restent sur ses genoux. Attends, je regarde. Mila s'arrête net. Maman attend, sans parler. Je regarde. Mila observe l'enveloppe, écoute la cuisine. Sur le rabat, un &lt;emphasis level="moderate"&gt;éclat d'enveloppe&lt;/emphasis&gt; luit. Là, près du rabat. Mila tient l'enveloppe des deux mains. Le papier est lisse, un peu tiède. Elle est tiède, papa. Tu la portes jusqu'à la porte ? Oui, papa. On avance ? Oui, maman. Mila aplatit le papier, sans forcer. Elle glisse l'enveloppe, très peu. Elle passe. Le rabat aussi, après. Victorina tend la main. Elle pousse un tout petit bord. Il y a une lettre ! C'est le soleil ! Je l'ouvre ? Oui, papa. La porte s'ouvre un peu. Ça sent la carotte chaude. Le soleil est pour moi ? Oui. Mila pose le crayon près du tiroir. Victorina pose la gomme rose.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Maman dit : on range. Amandine met une tasse dans la boîte. Nora met la cuillère.&lt;/slow&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Mila pousse l'enveloppe trop vite. Je la glisse, d'un coup ! Le papier se plie sous la porte. L'enveloppe reste coincée. Oh. Le soleil ne passe pas. Je la prends ! Mila avance la main vers Victorina. Tu l'attends, Mila ? Victorina ne bouge pas. Ses mains restent sur ses genoux. Attends, je regarde. Mila s'arrête net. Maman attend, sans parler. Je regarde. Mila observe l'enveloppe, écoute la cuisine. Sur le rabat, un &lt;emphasis&gt;éclat d'enveloppe&lt;/emphasis&gt; luit. Là, près du rabat. Mila tient l'enveloppe des deux mains. Le papier est lisse, un peu tiède. Elle est tiède, papa. Tu la portes jusqu'à la porte ? Oui, papa. On avance ? Oui, maman. Mila aplatit le papier, sans forcer. Elle glisse l'enveloppe, très peu. Elle passe. Le rabat aussi, après. Victorina tend la main. Elle pousse un tout petit bord. Il y a une lettre ! C'est le soleil ! Je l'ouvre ? Oui, papa. La porte s'ouvre un peu. Ça sent la carotte chaude. Le soleil est pour moi ? Oui. Mila pose le crayon près du tiroir. Victorina pose la gomme rose.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1841,30 +1876,34 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1873,28 +1912,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat d'enveloppe</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1903,36 +1946,73 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat_d_enveloppe; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|On range le crayon ?
+          <t>narrateur|Mila pousse l'enveloppe trop vite.
+enfant-f|Je la glisse, d'un coup !
+narrateur|Le papier se plie sous la porte.
+narrateur|L'enveloppe reste coincée.
+enfant-f|Oh.
+narrateur|Le soleil ne passe pas.
+enfant-f|Je la prends !
+narrateur|Mila avance la main vers Victorina.
+maman|Tu l'attends, Mila ?
+narrateur|Victorina ne bouge pas.
+narrateur|Ses mains restent sur ses genoux.
+enfant-f|Attends, je regarde.
+narrateur|Mila s'arrête net.
+narrateur|Maman attend, sans parler.
+enfant-f|Je regarde.
+narrateur|Mila observe l'enveloppe, écoute la cuisine.
+narrateur|Sur le rabat, un éclat d'enveloppe luit.
+enfant-f|Là, près du rabat.
+narrateur|Mila tient l'enveloppe des deux mains.
+narrateur|Le papier est lisse, un peu tiède.
+enfant-f|Elle est tiède, papa.
+papa|Tu la portes jusqu'à la porte ?
+enfant-f|Oui, papa.
+maman|On avance ?
+enfant-f|Oui, maman.
+narrateur|Mila aplatit le papier, sans forcer.
+narrateur|Elle glisse l'enveloppe, très peu.
+enfant-f|Elle passe.
+copine|Le rabat aussi, après.
+narrateur|Victorina tend la main.
+narrateur|Elle pousse un tout petit bord.
+papa|Il y a une lettre !
+enfant-f|C'est le soleil !
+papa|Je l'ouvre ?
+enfant-f|Oui, papa.
+narrateur|La porte s'ouvre un peu.
+narrateur|Ça sent la carotte chaude.
+papa|Le soleil est pour moi ?
 enfant-f|Oui.
-narrateur|Mila pose le crayon.
-narrateur|Victorina pose la gomme.
-narrateur|Le tiroir sent encore le papier.
-papa|Le soleil est sur la table.
-papa|Près des carottes.
-enfant-f|Il brille un peu.
-maman|Tu as fini de ranger ?
-enfant-f|Oui, maman.
-narrateur|Le rayon a bougé.
-narrateur|Il touche maintenant le tapis.
-narrateur|La cuisine sent la soupe.</t>
+narrateur|Mila pose le crayon près du tiroir.
+narrateur|Victorina pose la gomme rose.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>papier,porte</t>
         </is>
       </c>
     </row>
@@ -1959,17 +2039,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai envoyé le soleil. Victorina a regardé. Bravo, Mila. Le soleil est à table. L'enveloppe est vide, maintenant.</t>
+          <t>L'enveloppe brillait, papa. Tu le vois, comme tout à l'heure ? Oui, sur le rabat. Mila pose le soleil près des carottes. On le garde près de nous ? Oui, maman. Ça sentait le papier. Le tiroir est là. L'enveloppe reste ouverte, vide. Mila respire, plus large. On reste un peu ? Oui. Les joues de Mila se réchauffent. Le crayon reste tiède sous la main. Le rayon a glissé sur le bureau. Il est pâle. Comme tout à l'heure ? Oui, maman. Le rabat est luisant, toi ? Un peu, papa. La gomme rose ne roule plus. Elle est tiède. On la laisse au bureau ? Oui. Un éclat d'enveloppe reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai envoyé le soleil. Victorina a regardé. Bravo, Mila. Le soleil est à table. L'enveloppe est vide, maintenant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'enveloppe brillait, papa. Tu le vois, comme tout à l'heure ? Oui, sur le rabat. Mila pose le soleil près des carottes. On le garde près de nous ? Oui, maman. Ça sentait le papier. Le tiroir est là. L'enveloppe reste ouverte, vide. Mila respire, plus large. On reste un peu ? Oui. Les joues de Mila se réchauffent. Le crayon reste tiède sous la main. Le rayon a glissé sur le bureau. Il est pâle. Comme tout à l'heure ? Oui, maman. Le rabat est luisant, toi ? Un peu, papa. La gomme rose ne roule plus. Elle est tiède. On la laisse au bureau ? Oui. Un &lt;emphasis level="moderate"&gt;éclat d'enveloppe&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'enveloppe brillait, papa. Tu le vois, comme tout à l'heure ? Oui, sur le rabat. Mila pose le soleil près des carottes. On le garde près de nous ? Oui, maman. Ça sentait le papier. Le tiroir est là. L'enveloppe reste ouverte, vide. Mila respire, plus large. On reste un peu ? Oui. Les joues de Mila se réchauffent. Le crayon reste tiède sous la main. Le rayon a glissé sur le bureau. Il est pâle. Comme tout à l'heure ? Oui, maman. Le rabat est luisant, toi ? Un peu, papa. La gomme rose ne roule plus. Elle est tiède. On la laisse au bureau ? Oui. Un &lt;emphasis&gt;éclat d'enveloppe&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2016,7 +2096,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2024,7 +2104,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2036,12 +2116,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2050,17 +2130,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat d'enveloppe</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2069,11 +2153,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2082,28 +2166,57 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_d_enveloppe_reste_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai envoyé le soleil.
-enfant-f|Victorina a regardé.
-maman|Bravo, Mila.
-papa|Le soleil est à table.
-narrateur|L'enveloppe est vide, maintenant.</t>
+          <t>enfant-f|L'enveloppe brillait, papa.
+papa|Tu le vois, comme tout à l'heure ?
+enfant-f|Oui, sur le rabat.
+narrateur|Mila pose le soleil près des carottes.
+maman|On le garde près de nous ?
+enfant-f|Oui, maman.
+enfant-f|Ça sentait le papier.
+maman|Le tiroir est là.
+narrateur|L'enveloppe reste ouverte, vide.
+narrateur|Mila respire, plus large.
+papa|On reste un peu ?
+enfant-f|Oui.
+narrateur|Les joues de Mila se réchauffent.
+narrateur|Le crayon reste tiède sous la main.
+narrateur|Le rayon a glissé sur le bureau.
+enfant-f|Il est pâle.
+maman|Comme tout à l'heure ?
+enfant-f|Oui, maman.
+papa|Le rabat est luisant, toi ?
+enfant-f|Un peu, papa.
+narrateur|La gomme rose ne roule plus.
+enfant-f|Elle est tiède.
+maman|On la laisse au bureau ?
+enfant-f|Oui.
+narrateur|Un éclat d'enveloppe reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>cuisine</t>
         </is>
       </c>
     </row>
@@ -2124,7 +2237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2202,6 +2315,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>